<commit_message>
chore: 4 bug fixed, regen xlsx, redact
</commit_message>
<xml_diff>
--- a/reports/LifeOS-QA-Report.xlsx
+++ b/reports/LifeOS-QA-Report.xlsx
@@ -3821,7 +3821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3831,7 +3831,8 @@
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3872,6 +3873,11 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>Resolusi</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>Ditemukan di</t>
         </is>
       </c>
@@ -3894,7 +3900,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -3915,6 +3921,11 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
+          <t>By design — README + swagger nyatakan PUT full-replace; UI kirim objek penuh</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
           <t>TC-TASK-04</t>
         </is>
       </c>
@@ -3937,7 +3948,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -3956,6 +3967,11 @@
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Field _ts dihapus dari dashboard_handler.go</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>TC-DASH-01</t>
         </is>
@@ -3979,7 +3995,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -4000,6 +4016,11 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
+          <t>Helper badRequest 400 invalid di ~40 bind failure (errors.go)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
           <t>TC-FIN-05</t>
         </is>
       </c>
@@ -4022,7 +4043,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -4043,6 +4064,11 @@
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Komponen Field (useId) + htmlFor/id semua form + aria-label; bukti e2e getByLabel</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>TC-GOAL-05</t>
         </is>

</xml_diff>

<commit_message>
chore: 61TC e2e26 date-drift proof regen
</commit_message>
<xml_diff>
--- a/reports/LifeOS-QA-Report.xlsx
+++ b/reports/LifeOS-QA-Report.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>75/75 assertions pass</t>
+          <t>74/75 assertions pass</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3677,6 +3677,269 @@
       <c r="J57" s="4" t="inlineStr">
         <is>
           <t>go test pass, service 83.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>TC-CAL-03</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Halaman kalender render + legenda</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka Kalender
+2. Lihat grid + legenda</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Bulan tampil, legenda ▸◎₿◆ ada</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Playwright e2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>TC-TRV-03</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Halaman travel lengkap</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Seed Bandung</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka Travel</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Trip + 4 itinerary + 4 packing tampil</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Playwright e2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>TC-DEC-03</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Halaman keputusan + tambah opsi</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka Keputusan
+2. Tambah opsi baru</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Ranking tampil, opsi baru muncul</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Playwright e2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>TC-AST-03</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Halaman aset 3 seksi</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka Aset</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Aset + wishlist + dokumen tampil</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Playwright e2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>TC-CTC-03</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Halaman relasi tambah kontak</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka Relasi
+2. Tambah kontak baru</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Kontak baru muncul di list</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Playwright e2e</t>
         </is>
       </c>
     </row>
@@ -3779,7 +4042,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>75/75 Pass</t>
+          <t>74/75 Pass</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -4123,7 +4386,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -4133,7 +4396,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>COUNTIF('Test Cases'!I2:I57,"Pass")</f>
+        <f>COUNTIF('Test Cases'!I2:I62,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4144,7 +4407,7 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>COUNTIF('Test Cases'!I2:I57,"Fail")</f>
+        <f>COUNTIF('Test Cases'!I2:I62,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4155,7 +4418,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>COUNTIF('Test Cases'!I2:I57,"Not Run")</f>
+        <f>COUNTIF('Test Cases'!I2:I62,"Not Run")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: evidence 75/75 regen
</commit_message>
<xml_diff>
--- a/reports/LifeOS-QA-Report.xlsx
+++ b/reports/LifeOS-QA-Report.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>74/75 assertions pass</t>
+          <t>75/75 assertions pass</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>74/75 Pass</t>
+          <t>75/75 Pass</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">

</xml_diff>